<commit_message>
Updated books excel file
</commit_message>
<xml_diff>
--- a/books.xlsx
+++ b/books.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RAKESH\Desktop\Github\LibraryManagementSystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE1088D8-B52E-47A1-AD3E-5DBD771B8686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38DBC1E8-00B7-4AE0-8231-A2564BDB5075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="314">
   <si>
     <t>Title</t>
   </si>
@@ -133,9 +133,6 @@
     <t>Good Condition</t>
   </si>
   <si>
-    <t>1984</t>
-  </si>
-  <si>
     <t>George Orwell</t>
   </si>
   <si>
@@ -812,13 +809,1296 @@
   </si>
   <si>
     <t>ACC-1049</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>The Great Gatsby is a classic American novel written by F. Scott Fitzgerald. Set in the 1920s, the story follows the mysterious millionaire Jay Gatsby and his deep love for Daisy Buchanan. Through themes of love, wealth, ambition, and the American Dream, the novel explores the glamour and emptiness of high society in America during the Jazz Age. It is widely regarded as one of the greatest works of American literature.</t>
+  </si>
+  <si>
+    <t>To Kill a Mockingbird is a famous novel written by Harper Lee. Set in the American South during the 1930s, the story is narrated by a young girl named Scout Finch. The novel explores themes of racial injustice, morality, compassion, and courage through the experiences of Scout and her father, Atticus Finch, a lawyer defending a Black man wrongly accused of a crime. The book is considered a timeless classic of modern American literature.</t>
+  </si>
+  <si>
+    <t>Written by George Orwell, 1984 is a dystopian novel set in a totalitarian society ruled by the Party and its leader, Big Brother. The story follows Winston Smith, a government employee who secretly rebels against constant surveillance, censorship, and thought control. As Winston searches for truth and freedom, he faces the terrifying power of an oppressive regime that manipulates history, language, and human emotions. The novel explores themes of authoritarianism, propaganda, individuality, and psychological control. Considered one of the greatest political novels ever written, 1984 remains highly influential and relevant in discussions about freedom, privacy, and government power.</t>
+  </si>
+  <si>
+    <t>Written by Jane Austen, Pride and Prejudice is a classic romantic novel set in early 19th-century England. The story follows Elizabeth Bennet, an intelligent and independent young woman, and her evolving relationship with the wealthy but reserved Mr. Darcy. Through misunderstandings, social expectations, and personal growth, the novel explores themes of love, marriage, class, pride, and prejudice. Known for its wit, humor, and memorable characters, the book provides a sharp commentary on society and relationships of its time. It remains one of the most beloved works of English literature and has inspired numerous film and television adaptations.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by J.D. Salinger, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Catcher in the Rye</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> follows Holden Caulfield, a rebellious teenager who leaves his boarding school and wanders through New York City. As he struggles with loneliness, confusion, and the transition into adulthood, Holden criticizes the “phoniness” of the world around him. The novel explores themes of identity, alienation, innocence, and mental health. Known for its unique narrative voice and emotional depth, the book became a landmark in modern American literature and continues to resonate with young readers worldwide.</t>
+    </r>
+  </si>
+  <si>
+    <t>Written by J.R.R. Tolkien, The Hobbit is a fantasy adventure about Bilbo Baggins, a peaceful hobbit who is unexpectedly drawn into a dangerous journey with a group of dwarves and the wizard Gandalf. Their mission is to reclaim treasure guarded by the dragon Smaug. During the adventure, Bilbo discovers courage, intelligence, and inner strength. The novel introduces readers to the magical world of Middle-earth and features memorable creatures such as trolls, elves, goblins, and Gollum. It is considered one of the greatest fantasy novels ever written.</t>
+  </si>
+  <si>
+    <t>Written by Aldous Huxley, Brave New World is a dystopian novel set in a futuristic society where people are genetically engineered and conditioned to live in social harmony. Citizens are controlled through technology, consumerism, and a happiness-inducing drug called soma. Individuality, emotions, and deep relationships are discouraged in favor of stability and pleasure. The novel examines themes of freedom, science, technology, and social control. Huxley’s powerful vision of a controlled society remains highly relevant in discussions about modern culture and technological influence.</t>
+  </si>
+  <si>
+    <t>Written by Paulo Coelho, The Alchemist tells the story of Santiago, a young shepherd who dreams of finding treasure near the Egyptian pyramids. Along his journey, he meets various people who teach him important lessons about destiny, spirituality, courage, and following one’s dreams. The novel encourages readers to pursue their “Personal Legend” and trust the journey of life. With its simple yet inspirational storytelling, the book has become an international bestseller and continues to inspire millions of readers around the world.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Yuval Noah Harari, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Sapiens</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> explores the complete history of humankind, from the emergence of early human species to the modern technological world. The book discusses major developments such as the Cognitive Revolution, Agricultural Revolution, and Scientific Revolution, explaining how humans built civilizations, religions, economies, and political systems. Harari combines history, anthropology, and philosophy to examine humanity’s achievements and challenges. The book became globally popular for its engaging style and thought-provoking analysis of how humans shaped the world throughout history.</t>
+    </r>
+  </si>
+  <si>
+    <t>Written by Daniel Kahneman, Thinking, Fast and Slow explains how human thinking works through two systems: System 1, which is fast, emotional, and intuitive, and System 2, which is slow, logical, and analytical. The book explores decision-making, cognitive biases, judgment errors, and human behavior using psychological research and real-life examples. It helps readers understand why people often make irrational choices and how better thinking can improve decisions in everyday life, business, and relationships. The book is widely respected for making complex psychological concepts easy to understand.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Ray Dalio, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Principles</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a nonfiction book that shares the life lessons and management philosophies developed by Dalio during his successful career as a businessman and investor. The book focuses on decision-making, leadership, teamwork, honesty, and achieving goals through clear principles and self-reflection. Dalio explains how learning from mistakes and maintaining transparency can help individuals and organizations grow successfully. Combining personal experiences with practical advice, the book has become popular among entrepreneurs, students, and professionals seeking personal and professional improvement.</t>
+    </r>
+  </si>
+  <si>
+    <t>Written by James Clear, Atomic Habits is a self-improvement book that explains how small daily habits can create significant long-term success. The book provides practical methods for building good habits, breaking bad ones, and improving consistency through simple behavioral changes. Clear introduces concepts such as habit stacking, identity-based habits, and the power of incremental improvement. Using scientific research and real-life examples, the book shows how tiny positive actions can produce remarkable results over time. It has become one of the most influential modern books on productivity and personal growth.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Alex Michaelides, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Silent Patient</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a psychological thriller centered on Alicia Berenson, a famous painter who suddenly shoots her husband and then refuses to speak another word. Theo Faber, a criminal psychotherapist, becomes obsessed with uncovering the truth behind her silence. As Theo investigates Alicia’s past, shocking secrets and unexpected twists begin to emerge. The novel explores themes of trauma, obsession, psychology, and deception. Known for its suspenseful storytelling and surprising ending, the book became an international bestseller and a favorite among thriller readers.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Frank Herbert, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Dune</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is an epic science fiction novel set in a distant future where noble families compete for control of the desert planet Arrakis. The story follows Paul Atreides, whose family becomes ruler of Arrakis, the only source of the valuable substance known as “spice.” As political conflict, betrayal, and war unfold, Paul discovers his extraordinary destiny. The novel explores themes of power, religion, ecology, survival, and human potential. Widely regarded as one of the greatest science fiction novels ever written, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Dune</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> has inspired films, television series, and modern sci-fi storytelling.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Isaac Asimov, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Foundation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a groundbreaking science fiction novel that follows mathematician Hari Seldon, who develops a science called psychohistory capable of predicting the future of large populations. Seldon foresees the collapse of the Galactic Empire and creates the Foundation to preserve knowledge and reduce the coming age of chaos. The story spans generations and explores politics, science, leadership, and civilization. Known for its ambitious ideas and intelligent storytelling, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Foundation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> became one of the most influential works in science fiction literature.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Markus Zusak, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Book Thief</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a historical novel set in Nazi Germany during World War II. Narrated by Death, the story follows a young girl named Liesel Meminger, who finds comfort in stealing books and sharing stories with others during difficult times. Living with foster parents and hiding a Jewish man in their basement, Liesel experiences love, friendship, fear, and loss amid the horrors of war. The novel explores themes of humanity, courage, words, and survival. It is praised for its emotional storytelling and unique narrative style.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Louisa May Alcott, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Little Women</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a coming-of-age novel that follows the lives of the four March sisters—Meg, Jo, Beth, and Amy—during the American Civil War. Each sister has a distinct personality and dreams for the future, and together they experience love, hardship, friendship, and personal growth. The novel explores themes of family, independence, sacrifice, and womanhood. Known for its warmth, emotional depth, and memorable characters, the book remains a beloved classic and has inspired many film and television adaptations.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Herman Melville, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Moby Dick</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tells the story of Captain Ahab’s obsessive pursuit of the giant white whale that previously destroyed his ship and injured him. Narrated by Ishmael, the novel combines adventure, philosophy, and detailed descriptions of whaling life. As Ahab’s obsession grows stronger, the crew of the Pequod faces increasing danger and tragedy. The book explores themes of revenge, fate, obsession, nature, and humanity’s struggle against powerful forces. Considered one of the greatest American novels, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Moby Dick</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is admired for its depth and symbolism.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Leo Tolstoy, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>War and Peace</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a monumental historical novel set during the Napoleonic Wars in early 19th-century Russia. The story follows several aristocratic families as they experience war, love, loss, and personal transformation. Combining fictional characters with real historical events, the novel explores themes of destiny, power, family, history, and human nature. Tolstoy presents both grand battle scenes and intimate emotional moments with remarkable detail and realism. Widely regarded as one of the greatest novels ever written, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>War and Peace</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> remains a masterpiece of world literature.</t>
+    </r>
+  </si>
+  <si>
+    <t>Written by James Joyce, Ulysses is a modernist masterpiece that follows Leopold Bloom through a single day in Dublin on June 16, 1904. Inspired by Homer’s The Odyssey, the novel explores ordinary life through complex literary techniques, stream-of-consciousness narration, and deep psychological insight. The book examines themes of identity, relationships, memory, and modern society. Known for its experimental style and intellectual depth, Ulysses is considered one of the greatest and most influential novels in world literature.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Homer, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Odyssey</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is an ancient Greek epic poem that tells the story of Odysseus and his ten-year journey home after the Trojan War. Along the way, he faces dangerous creatures, powerful gods, and difficult challenges while his wife Penelope and son Telemachus wait for his return. The poem explores themes of bravery, loyalty, intelligence, and perseverance. It remains one of the most important works of classical literature and has influenced storytelling for centuries.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Fyodor Dostoevsky, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Crime and Punishment</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> follows Rodion Raskolnikov, a poor former student who murders a pawnbroker believing he is morally justified. After the crime, he struggles with guilt, fear, and psychological torment. The novel explores themes of morality, justice, redemption, and human suffering. Through intense psychological analysis and philosophical discussions, Dostoevsky examines the consequences of crime on the human mind. The book is regarded as one of the greatest psychological novels ever written.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Fyodor Dostoevsky, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Brothers Karamazov</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a philosophical novel centered on the conflict between three brothers and their immoral father. The story explores themes of faith, free will, morality, justice, and family relationships. Each brother represents different aspects of human nature and philosophical thought. Through murder, emotional conflict, and spiritual questioning, the novel examines the struggle between good and evil. It is considered one of the greatest achievements in world literature for its emotional intensity and intellectual depth.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Leo Tolstoy, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Anna Karenina</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tells the tragic story of Anna, a married aristocratic woman who falls passionately in love with Count Vronsky. Their affair leads to emotional conflict, social judgment, and personal tragedy. Alongside Anna’s story, the novel follows Konstantin Levin’s search for meaning, faith, and happiness. The book explores themes of love, marriage, society, morality, and family life in 19th-century Russia. Widely praised for its realism and psychological depth, it is regarded as one of the greatest novels ever written.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Dante Alighieri, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Divine Comedy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is an epic poem describing a spiritual journey through Hell, Purgatory, and Heaven. Guided first by the Roman poet Virgil and later by Beatrice, Dante witnesses the consequences of sin and the path toward salvation. The poem explores themes of justice, morality, faith, and redemption while presenting vivid descriptions of the afterlife. Considered a masterpiece of Italian literature, the work has greatly influenced religion, philosophy, and Western culture.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Homer, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Iliad</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is an ancient Greek epic poem set during the Trojan War. The story focuses on the anger of the warrior Achilles after a conflict with King Agamemnon. As battles rage between the Greeks and Trojans, the poem explores themes of honor, pride, fate, heroism, and mortality. Featuring legendary heroes such as Hector and Achilles, the epic remains one of the most important works of classical literature and has shaped Western storytelling for centuries.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by William Shakespeare, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hamlet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a tragic play about Prince Hamlet of Denmark, who seeks revenge after learning that his uncle Claudius murdered his father and seized the throne. Struggling with grief, anger, and uncertainty, Hamlet questions morality, life, and death. The play explores themes of revenge, madness, betrayal, and existential thought. Famous for lines such as “To be, or not to be,” </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hamlet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is regarded as one of Shakespeare’s greatest works and a masterpiece of world drama.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by William Shakespeare, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Macbeth</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tells the story of a Scottish general who becomes consumed by ambition after hearing a prophecy that he will become king. Encouraged by Lady Macbeth, he murders King Duncan and takes the throne. As guilt and paranoia grow, Macbeth descends into tyranny and violence. The play explores themes of ambition, power, fate, guilt, and corruption. Known for its dark atmosphere and dramatic intensity, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Macbeth</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> remains one of Shakespeare’s most famous tragedies.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by William Shakespeare, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Othello</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a tragic play about a respected military general who is manipulated by his jealous officer, Iago. Through lies and deception, Iago convinces Othello that his wife Desdemona has been unfaithful. Consumed by jealousy and anger, Othello makes devastating decisions that lead to tragedy. The play explores themes of jealousy, trust, racism, betrayal, and manipulation. It is considered one of Shakespeare’s most powerful and emotionally intense dramas.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by William Shakespeare, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Tempest</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> follows Prospero, the rightful Duke of Milan, who lives on a remote island after being betrayed by his brother. Using magical powers, Prospero creates a storm that brings his enemies to the island, allowing him to seek justice and reconciliation. The play explores themes of forgiveness, power, revenge, freedom, and magic. Often considered Shakespeare’s final play, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Tempest</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is admired for its imaginative storytelling and emotional depth.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Mary Shelley, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Frankenstein</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tells the story of Victor Frankenstein, a scientist who creates a living creature through scientific experimentation. Horrified by his creation, Victor abandons the creature, which later seeks revenge after suffering loneliness and rejection. The novel explores themes of ambition, responsibility, science, isolation, and humanity. Considered one of the first science fiction novels, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Frankenstein</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> remains influential for its exploration of the dangers of unchecked scientific ambition.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Bram Stoker, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Dracula</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a gothic horror novel about Count Dracula, a vampire who travels from Transylvania to England in search of new victims. Told through letters and diary entries, the story follows a group led by Professor Van Helsing as they attempt to stop Dracula’s evil plans. The novel explores themes of fear, immortality, superstition, and good versus evil. It became one of the most famous horror novels ever written and established many modern vampire traditions.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Oscar Wilde, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Picture of Dorian Gray</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tells the story of a handsome young man who wishes to remain forever young while his portrait ages instead. As Dorian pursues pleasure and immoral behavior, the portrait reflects the corruption of his soul. The novel explores themes of vanity, beauty, morality, art, and temptation. Known for its wit and philosophical ideas, the book remains a classic exploration of human desire and the consequences of selfish living.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Franz Kafka, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Metamorphosis</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> begins when Gregor Samsa wakes up transformed into a giant insect. Unable to work or communicate properly, Gregor becomes isolated from his family and society. The novella explores themes of alienation, identity, guilt, and human relationships. Kafka’s surreal storytelling and psychological depth create a powerful examination of loneliness and the struggle for acceptance. The work is considered one of the most influential pieces of modern literature.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Emily Brontë, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wuthering Heights</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a dark and passionate novel about the intense relationship between Heathcliff and Catherine Earnshaw. Their love is filled with obsession, revenge, jealousy, and emotional conflict, affecting multiple generations. Set on the wild Yorkshire moors, the novel explores themes of love, hatred, social class, and revenge. Its gothic atmosphere and complex characters have made it one of the most famous works in English literature.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Charlotte Brontë, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Jane Eyre</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> follows the life of an orphaned girl who grows into an intelligent and independent woman. Jane becomes a governess at Thornfield Hall, where she falls in love with her mysterious employer, Mr. Rochester. As secrets about Rochester emerge, Jane must choose between love and her personal values. The novel explores themes of love, morality, independence, religion, and social class. It remains a celebrated classic for its emotional strength and strong female protagonist.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Charles Dickens, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Great Expectations</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a coming-of-age novel that follows the life of Pip, an orphan boy raised by his strict sister. After receiving unexpected financial support from a mysterious benefactor, Pip moves to London and enters high society. As he pursues wealth, education, and love, he learns important lessons about ambition, loyalty, and personal values. The novel explores themes of social class, identity, guilt, and personal growth. It is regarded as one of Dickens’s greatest literary achievements.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Charles Dickens, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A Tale of Two Cities</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is set during the French Revolution in London and Paris. The story follows Charles Darnay, a French aristocrat, and Sydney Carton, a troubled English lawyer, whose lives become connected through love and sacrifice. As political violence and revolution spread across France, the novel explores themes of justice, revenge, resurrection, and social inequality. Famous for its opening line, “It was the best of times, it was the worst of times,” the book remains one of Dickens’s most celebrated historical novels.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Charles Dickens, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Oliver Twist</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tells the story of a poor orphan boy who escapes from a harsh workhouse and travels to London. There, he becomes involved with a gang of young thieves led by the criminal Fagin. Despite facing poverty, crime, and exploitation, Oliver maintains his innocence and kindness. The novel explores themes of social injustice, childhood suffering, crime, and compassion. Through memorable characters and emotional storytelling, Dickens criticized the treatment of poor children in Victorian England.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Victor Hugo, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Les Misérables</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is an epic novel about redemption, justice, and social inequality in 19th-century France. The story follows Jean Valjean, a former prisoner trying to rebuild his life while being relentlessly pursued by Inspector Javert. Alongside political unrest and personal struggles, the novel explores themes of mercy, love, sacrifice, poverty, and revolution. Known for its emotional depth and unforgettable characters, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Les Misérables</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is considered one of the greatest works of world literature and has inspired famous stage and film adaptations.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Victor Hugo, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Hunchback of Notre-Dame</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a gothic novel set in medieval Paris. The story centers on Quasimodo, the deformed bell-ringer of Notre-Dame Cathedral, and his tragic connection with the kind-hearted dancer Esmeralda. As jealousy, obsession, and injustice unfold, the novel explores themes of love, social rejection, fate, and compassion. Hugo also highlights the beauty and importance of Gothic architecture through vivid descriptions of Paris and the cathedral itself.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Alexandre Dumas, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Count of Monte Cristo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> follows Edmond Dantès, a young sailor falsely imprisoned because of betrayal and jealousy. After escaping prison and discovering hidden treasure, he transforms himself into the wealthy Count of Monte Cristo and carefully plans revenge against those who destroyed his life. The novel explores themes of justice, revenge, forgiveness, and hope. Filled with adventure, suspense, and dramatic twists, it remains one of the most popular and influential adventure novels ever written.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Alexandre Dumas, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Three Musketeers</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is an adventure novel about a young man named d’Artagnan who travels to Paris hoping to join the King’s Musketeers. He befriends Athos, Porthos, and Aramis, and together they become involved in political conspiracies, dangerous missions, and heroic battles. The novel explores themes of friendship, loyalty, honor, and bravery. Famous for the phrase “All for one, and one for all,” the story remains a timeless classic of historical adventure fiction.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Miguel de Cervantes, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Don Quixote</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> follows an aging Spanish nobleman who becomes obsessed with stories of knights and decides to become a wandering knight himself. Accompanied by his loyal squire Sancho Panza, Don Quixote embarks on humorous adventures, often confusing imagination with reality. The novel explores themes of idealism, madness, literature, and human nature. Widely considered one of the greatest novels ever written, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Don Quixote</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is admired for its humor, creativity, and influence on modern fiction.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Gustave Flaubert, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Madame Bovary</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tells the story of Emma Bovary, a woman dissatisfied with her ordinary life and marriage. Seeking excitement and romance, she becomes involved in affairs and spends beyond her means, leading to emotional and financial disaster. The novel explores themes of desire, boredom, social expectations, and the conflict between dreams and reality. Known for its realistic style and psychological depth, the book became one of the most influential novels in literary realism.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Albert Camus, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The Stranger</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> follows Meursault, an emotionally detached man living in French Algeria. After committing a senseless murder, he faces trial and judgment not only for the crime but also for his indifference toward life and society. The novel explores themes of absurdism, alienation, death, and the search for meaning in an indifferent universe. Camus’s simple yet powerful writing style made the book a major work of existential and philosophical literature.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Ray Bradbury, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fahrenheit 451</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a dystopian novel set in a future society where books are banned and “firemen” burn any books they find. The story follows Guy Montag, a fireman who begins questioning his role after meeting people who value literature and free thought. As Montag secretly starts reading books, he rebels against a society controlled by censorship and entertainment. The novel explores themes of knowledge, freedom, censorship, and individuality. It remains a classic warning about the dangers of suppressing ideas and critical thinking.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by George Orwell, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Animal Farm</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a political allegory in which farm animals overthrow their human owner to create an equal society. However, the pigs gradually seize power and establish a dictatorship even more oppressive than before. The novella satirizes the Russian Revolution and the corruption of political ideals. Through simple storytelling and memorable characters, Orwell explores themes of power, propaganda, inequality, and betrayal. The book remains one of the most influential political satires ever written.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by William Golding, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Lord of the Flies</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tells the story of a group of schoolboys stranded on a deserted island after a plane crash. Initially attempting to build a civilized society, the boys gradually descend into fear, violence, and savagery. The novel explores themes of human nature, power, civilization, fear, and morality. Through the boys’ struggle for survival, Golding presents a dark view of humanity and the fragile nature of social order. The book is regarded as a classic of modern literature.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Written by Gabriel García Márquez, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>One Hundred Years of Solitude</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is a landmark work of magical realism that tells the multi-generational story of the Buendía family in the fictional town of Macondo. Combining reality with magical and supernatural events, the novel explores themes of love, solitude, destiny, memory, and the passage of time. Through richly imaginative storytelling and symbolic characters, Márquez portrays the rise and decline of both a family and a society. The book is widely regarded as one of the greatest masterpieces of world literature.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -831,6 +2111,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -847,7 +2135,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -870,16 +2158,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1184,7 +2504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:P51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1202,7 +2522,7 @@
     <col min="15" max="15" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1248,8 +2568,11 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="3" t="s">
+        <v>263</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
@@ -1295,8 +2618,11 @@
       <c r="O2" s="2">
         <v>15.99</v>
       </c>
+      <c r="P2" s="4" t="s">
+        <v>264</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>27</v>
       </c>
@@ -1342,16 +2668,19 @@
       <c r="O3" s="2">
         <v>16.989999999999998</v>
       </c>
+      <c r="P3" s="4" t="s">
+        <v>265</v>
+      </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>1984</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>18</v>
@@ -1360,13 +2689,13 @@
         <v>2002</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>22</v>
@@ -1375,10 +2704,10 @@
         <v>33</v>
       </c>
       <c r="K4" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L4" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="M4" s="2">
         <v>3</v>
@@ -1389,16 +2718,19 @@
       <c r="O4" s="2">
         <v>17.989999999999998</v>
       </c>
+      <c r="P4" s="4" t="s">
+        <v>266</v>
+      </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>30</v>
@@ -1407,13 +2739,13 @@
         <v>2003</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>22</v>
@@ -1422,10 +2754,10 @@
         <v>23</v>
       </c>
       <c r="K5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L5" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="M5" s="2">
         <v>4</v>
@@ -1436,16 +2768,19 @@
       <c r="O5" s="2">
         <v>18.989999999999998</v>
       </c>
+      <c r="P5" s="4" t="s">
+        <v>267</v>
+      </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>53</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>18</v>
@@ -1454,13 +2789,13 @@
         <v>2004</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>22</v>
@@ -1469,10 +2804,10 @@
         <v>33</v>
       </c>
       <c r="K6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="L6" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="M6" s="2">
         <v>5</v>
@@ -1483,16 +2818,19 @@
       <c r="O6" s="2">
         <v>19.989999999999998</v>
       </c>
+      <c r="P6" t="s">
+        <v>268</v>
+      </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>60</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>30</v>
@@ -1507,7 +2845,7 @@
         <v>20</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>22</v>
@@ -1516,10 +2854,10 @@
         <v>33</v>
       </c>
       <c r="K7" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="L7" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>63</v>
       </c>
       <c r="M7" s="2">
         <v>1</v>
@@ -1530,16 +2868,19 @@
       <c r="O7" s="2">
         <v>20.99</v>
       </c>
+      <c r="P7" s="5" t="s">
+        <v>269</v>
+      </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>18</v>
@@ -1554,7 +2895,7 @@
         <v>20</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>22</v>
@@ -1563,10 +2904,10 @@
         <v>23</v>
       </c>
       <c r="K8" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="L8" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="M8" s="2">
         <v>2</v>
@@ -1577,16 +2918,19 @@
       <c r="O8" s="2">
         <v>21.99</v>
       </c>
+      <c r="P8" s="5" t="s">
+        <v>270</v>
+      </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>72</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>30</v>
@@ -1595,13 +2939,13 @@
         <v>2007</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>22</v>
@@ -1610,10 +2954,10 @@
         <v>33</v>
       </c>
       <c r="K9" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="L9" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>75</v>
       </c>
       <c r="M9" s="2">
         <v>3</v>
@@ -1624,16 +2968,19 @@
       <c r="O9" s="2">
         <v>22.99</v>
       </c>
+      <c r="P9" s="5" t="s">
+        <v>271</v>
+      </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>78</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>18</v>
@@ -1642,13 +2989,13 @@
         <v>2008</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>22</v>
@@ -1657,10 +3004,10 @@
         <v>33</v>
       </c>
       <c r="K10" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="L10" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>81</v>
       </c>
       <c r="M10" s="2">
         <v>4</v>
@@ -1671,16 +3018,19 @@
       <c r="O10" s="2">
         <v>23.99</v>
       </c>
+      <c r="P10" t="s">
+        <v>272</v>
+      </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>84</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>30</v>
@@ -1689,13 +3039,13 @@
         <v>2009</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>22</v>
@@ -1704,10 +3054,10 @@
         <v>23</v>
       </c>
       <c r="K11" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="L11" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="M11" s="2">
         <v>5</v>
@@ -1718,16 +3068,19 @@
       <c r="O11" s="2">
         <v>24.99</v>
       </c>
+      <c r="P11" s="5" t="s">
+        <v>273</v>
+      </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>90</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>18</v>
@@ -1742,7 +3095,7 @@
         <v>20</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>22</v>
@@ -1751,10 +3104,10 @@
         <v>33</v>
       </c>
       <c r="K12" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="L12" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="M12" s="2">
         <v>1</v>
@@ -1765,16 +3118,19 @@
       <c r="O12" s="2">
         <v>25.99</v>
       </c>
+      <c r="P12" t="s">
+        <v>274</v>
+      </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>30</v>
@@ -1789,7 +3145,7 @@
         <v>20</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>22</v>
@@ -1798,10 +3154,10 @@
         <v>33</v>
       </c>
       <c r="K13" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="L13" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>99</v>
       </c>
       <c r="M13" s="2">
         <v>2</v>
@@ -1812,16 +3168,19 @@
       <c r="O13" s="2">
         <v>26.99</v>
       </c>
+      <c r="P13" s="5" t="s">
+        <v>275</v>
+      </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>18</v>
@@ -1830,13 +3189,13 @@
         <v>2012</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>22</v>
@@ -1845,10 +3204,10 @@
         <v>23</v>
       </c>
       <c r="K14" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="L14" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>105</v>
       </c>
       <c r="M14" s="2">
         <v>3</v>
@@ -1859,16 +3218,19 @@
       <c r="O14" s="2">
         <v>27.99</v>
       </c>
+      <c r="P14" t="s">
+        <v>276</v>
+      </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>30</v>
@@ -1877,13 +3239,13 @@
         <v>2013</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>22</v>
@@ -1892,10 +3254,10 @@
         <v>33</v>
       </c>
       <c r="K15" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="L15" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>111</v>
       </c>
       <c r="M15" s="2">
         <v>4</v>
@@ -1906,16 +3268,19 @@
       <c r="O15" s="2">
         <v>28.99</v>
       </c>
+      <c r="P15" t="s">
+        <v>277</v>
+      </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>18</v>
@@ -1924,13 +3289,13 @@
         <v>2014</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>22</v>
@@ -1939,10 +3304,10 @@
         <v>33</v>
       </c>
       <c r="K16" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="L16" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="M16" s="2">
         <v>5</v>
@@ -1953,16 +3318,19 @@
       <c r="O16" s="2">
         <v>29.99</v>
       </c>
+      <c r="P16" t="s">
+        <v>278</v>
+      </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>120</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>30</v>
@@ -1977,7 +3345,7 @@
         <v>20</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>22</v>
@@ -1986,10 +3354,10 @@
         <v>23</v>
       </c>
       <c r="K17" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="L17" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="M17" s="2">
         <v>1</v>
@@ -2000,16 +3368,19 @@
       <c r="O17" s="2">
         <v>30.99</v>
       </c>
+      <c r="P17" t="s">
+        <v>279</v>
+      </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>18</v>
@@ -2033,10 +3404,10 @@
         <v>33</v>
       </c>
       <c r="K18" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="L18" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="L18" s="2" t="s">
-        <v>128</v>
       </c>
       <c r="M18" s="2">
         <v>2</v>
@@ -2047,16 +3418,19 @@
       <c r="O18" s="2">
         <v>31.99</v>
       </c>
+      <c r="P18" t="s">
+        <v>280</v>
+      </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>131</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>30</v>
@@ -2065,7 +3439,7 @@
         <v>2017</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>20</v>
@@ -2080,10 +3454,10 @@
         <v>33</v>
       </c>
       <c r="K19" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="L19" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="L19" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="M19" s="2">
         <v>3</v>
@@ -2094,16 +3468,19 @@
       <c r="O19" s="2">
         <v>32.99</v>
       </c>
+      <c r="P19" t="s">
+        <v>281</v>
+      </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>136</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>18</v>
@@ -2112,13 +3489,13 @@
         <v>2018</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>22</v>
@@ -2127,10 +3504,10 @@
         <v>23</v>
       </c>
       <c r="K20" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="L20" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="L20" s="2" t="s">
-        <v>138</v>
       </c>
       <c r="M20" s="2">
         <v>4</v>
@@ -2141,16 +3518,19 @@
       <c r="O20" s="2">
         <v>33.99</v>
       </c>
+      <c r="P20" t="s">
+        <v>282</v>
+      </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>30</v>
@@ -2159,13 +3539,13 @@
         <v>2019</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>22</v>
@@ -2174,10 +3554,10 @@
         <v>33</v>
       </c>
       <c r="K21" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="L21" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>143</v>
       </c>
       <c r="M21" s="2">
         <v>5</v>
@@ -2188,16 +3568,19 @@
       <c r="O21" s="2">
         <v>34.99</v>
       </c>
+      <c r="P21" s="6" t="s">
+        <v>283</v>
+      </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>18</v>
@@ -2212,7 +3595,7 @@
         <v>20</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>22</v>
@@ -2221,10 +3604,10 @@
         <v>33</v>
       </c>
       <c r="K22" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="L22" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="L22" s="2" t="s">
-        <v>148</v>
       </c>
       <c r="M22" s="2">
         <v>1</v>
@@ -2235,16 +3618,19 @@
       <c r="O22" s="2">
         <v>35.99</v>
       </c>
+      <c r="P22" t="s">
+        <v>284</v>
+      </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>151</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>30</v>
@@ -2259,7 +3645,7 @@
         <v>20</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>22</v>
@@ -2268,10 +3654,10 @@
         <v>23</v>
       </c>
       <c r="K23" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="L23" s="2" t="s">
         <v>152</v>
-      </c>
-      <c r="L23" s="2" t="s">
-        <v>153</v>
       </c>
       <c r="M23" s="2">
         <v>2</v>
@@ -2282,16 +3668,19 @@
       <c r="O23" s="2">
         <v>36.99</v>
       </c>
+      <c r="P23" t="s">
+        <v>285</v>
+      </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>155</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>18</v>
@@ -2300,13 +3689,13 @@
         <v>2022</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>22</v>
@@ -2315,10 +3704,10 @@
         <v>33</v>
       </c>
       <c r="K24" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="L24" s="2" t="s">
         <v>156</v>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>157</v>
       </c>
       <c r="M24" s="2">
         <v>3</v>
@@ -2329,16 +3718,19 @@
       <c r="O24" s="2">
         <v>37.99</v>
       </c>
+      <c r="P24" t="s">
+        <v>286</v>
+      </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>158</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>159</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>30</v>
@@ -2347,13 +3739,13 @@
         <v>2023</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>22</v>
@@ -2362,10 +3754,10 @@
         <v>33</v>
       </c>
       <c r="K25" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="L25" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>161</v>
       </c>
       <c r="M25" s="2">
         <v>4</v>
@@ -2376,16 +3768,19 @@
       <c r="O25" s="2">
         <v>38.99</v>
       </c>
+      <c r="P25" t="s">
+        <v>287</v>
+      </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>164</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>18</v>
@@ -2394,13 +3789,13 @@
         <v>2000</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>22</v>
@@ -2409,10 +3804,10 @@
         <v>23</v>
       </c>
       <c r="K26" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="L26" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>166</v>
       </c>
       <c r="M26" s="2">
         <v>5</v>
@@ -2423,16 +3818,19 @@
       <c r="O26" s="2">
         <v>39.99</v>
       </c>
+      <c r="P26" t="s">
+        <v>288</v>
+      </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>168</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>30</v>
@@ -2447,7 +3845,7 @@
         <v>20</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>22</v>
@@ -2456,10 +3854,10 @@
         <v>33</v>
       </c>
       <c r="K27" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="L27" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>170</v>
       </c>
       <c r="M27" s="2">
         <v>1</v>
@@ -2470,16 +3868,19 @@
       <c r="O27" s="2">
         <v>40.99</v>
       </c>
+      <c r="P27" t="s">
+        <v>289</v>
+      </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>172</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>173</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>18</v>
@@ -2494,7 +3895,7 @@
         <v>20</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>22</v>
@@ -2503,10 +3904,10 @@
         <v>33</v>
       </c>
       <c r="K28" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="L28" s="2" t="s">
         <v>174</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>175</v>
       </c>
       <c r="M28" s="2">
         <v>2</v>
@@ -2517,16 +3918,19 @@
       <c r="O28" s="2">
         <v>41.99</v>
       </c>
+      <c r="P28" t="s">
+        <v>290</v>
+      </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>177</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>30</v>
@@ -2535,13 +3939,13 @@
         <v>2003</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>22</v>
@@ -2550,10 +3954,10 @@
         <v>23</v>
       </c>
       <c r="K29" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="L29" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="L29" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="M29" s="2">
         <v>3</v>
@@ -2564,16 +3968,19 @@
       <c r="O29" s="2">
         <v>42.99</v>
       </c>
+      <c r="P29" t="s">
+        <v>291</v>
+      </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>180</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>181</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>18</v>
@@ -2582,13 +3989,13 @@
         <v>2004</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>22</v>
@@ -2597,10 +4004,10 @@
         <v>33</v>
       </c>
       <c r="K30" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="L30" s="2" t="s">
         <v>182</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>183</v>
       </c>
       <c r="M30" s="2">
         <v>4</v>
@@ -2611,16 +4018,19 @@
       <c r="O30" s="2">
         <v>43.99</v>
       </c>
+      <c r="P30" t="s">
+        <v>292</v>
+      </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>184</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>185</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>30</v>
@@ -2629,13 +4039,13 @@
         <v>2005</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>22</v>
@@ -2644,10 +4054,10 @@
         <v>33</v>
       </c>
       <c r="K31" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="L31" s="2" t="s">
         <v>186</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>187</v>
       </c>
       <c r="M31" s="2">
         <v>5</v>
@@ -2658,16 +4068,19 @@
       <c r="O31" s="2">
         <v>44.99</v>
       </c>
+      <c r="P31" t="s">
+        <v>293</v>
+      </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>189</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>190</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>18</v>
@@ -2682,7 +4095,7 @@
         <v>20</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I32" s="2" t="s">
         <v>22</v>
@@ -2691,7 +4104,7 @@
         <v>23</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="L32" s="2" t="s">
         <v>25</v>
@@ -2705,16 +4118,19 @@
       <c r="O32" s="2">
         <v>45.99</v>
       </c>
+      <c r="P32" t="s">
+        <v>294</v>
+      </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>194</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>30</v>
@@ -2729,7 +4145,7 @@
         <v>20</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>22</v>
@@ -2738,7 +4154,7 @@
         <v>33</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="L33" s="2" t="s">
         <v>35</v>
@@ -2752,16 +4168,19 @@
       <c r="O33" s="2">
         <v>46.99</v>
       </c>
+      <c r="P33" t="s">
+        <v>295</v>
+      </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>197</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>198</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>18</v>
@@ -2770,7 +4189,7 @@
         <v>2008</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>20</v>
@@ -2785,10 +4204,10 @@
         <v>33</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M34" s="2">
         <v>3</v>
@@ -2799,16 +4218,19 @@
       <c r="O34" s="2">
         <v>47.99</v>
       </c>
+      <c r="P34" t="s">
+        <v>296</v>
+      </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>201</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>202</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>30</v>
@@ -2817,7 +4239,7 @@
         <v>2009</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>20</v>
@@ -2832,10 +4254,10 @@
         <v>23</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="M35" s="2">
         <v>4</v>
@@ -2846,16 +4268,19 @@
       <c r="O35" s="2">
         <v>48.99</v>
       </c>
+      <c r="P35" t="s">
+        <v>297</v>
+      </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>206</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>18</v>
@@ -2864,13 +4289,13 @@
         <v>2010</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>22</v>
@@ -2879,10 +4304,10 @@
         <v>33</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M36" s="2">
         <v>5</v>
@@ -2893,16 +4318,19 @@
       <c r="O36" s="2">
         <v>49.99</v>
       </c>
+      <c r="P36" t="s">
+        <v>298</v>
+      </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>209</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>210</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>30</v>
@@ -2917,7 +4345,7 @@
         <v>20</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>22</v>
@@ -2926,10 +4354,10 @@
         <v>33</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M37" s="2">
         <v>1</v>
@@ -2940,16 +4368,19 @@
       <c r="O37" s="2">
         <v>50.99</v>
       </c>
+      <c r="P37" t="s">
+        <v>299</v>
+      </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>213</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>214</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>18</v>
@@ -2964,7 +4395,7 @@
         <v>20</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>22</v>
@@ -2973,10 +4404,10 @@
         <v>23</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M38" s="2">
         <v>2</v>
@@ -2987,16 +4418,19 @@
       <c r="O38" s="2">
         <v>51.99</v>
       </c>
+      <c r="P38" t="s">
+        <v>300</v>
+      </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>216</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>217</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>30</v>
@@ -3005,13 +4439,13 @@
         <v>2013</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>22</v>
@@ -3020,10 +4454,10 @@
         <v>33</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="M39" s="2">
         <v>3</v>
@@ -3034,16 +4468,19 @@
       <c r="O39" s="2">
         <v>52.99</v>
       </c>
+      <c r="P39" t="s">
+        <v>301</v>
+      </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>219</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>220</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>18</v>
@@ -3052,13 +4489,13 @@
         <v>2014</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>22</v>
@@ -3067,10 +4504,10 @@
         <v>33</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="M40" s="2">
         <v>4</v>
@@ -3081,16 +4518,19 @@
       <c r="O40" s="2">
         <v>53.99</v>
       </c>
+      <c r="P40" t="s">
+        <v>302</v>
+      </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="C41" s="2" t="s">
         <v>223</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>224</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>30</v>
@@ -3099,13 +4539,13 @@
         <v>2015</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I41" s="2" t="s">
         <v>22</v>
@@ -3114,10 +4554,10 @@
         <v>23</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="M41" s="2">
         <v>5</v>
@@ -3128,16 +4568,19 @@
       <c r="O41" s="2">
         <v>54.99</v>
       </c>
+      <c r="P41" t="s">
+        <v>303</v>
+      </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>226</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>227</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>18</v>
@@ -3152,19 +4595,19 @@
         <v>20</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J42" s="2" t="s">
         <v>33</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="M42" s="2">
         <v>1</v>
@@ -3175,16 +4618,19 @@
       <c r="O42" s="2">
         <v>55.99</v>
       </c>
+      <c r="P42" t="s">
+        <v>304</v>
+      </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="C43" s="2" t="s">
         <v>231</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>232</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>30</v>
@@ -3199,19 +4645,19 @@
         <v>20</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J43" s="2" t="s">
         <v>33</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M43" s="2">
         <v>2</v>
@@ -3222,16 +4668,19 @@
       <c r="O43" s="2">
         <v>56.99</v>
       </c>
+      <c r="P43" t="s">
+        <v>305</v>
+      </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>234</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>235</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>18</v>
@@ -3240,25 +4689,25 @@
         <v>2018</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J44" s="2" t="s">
         <v>23</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M44" s="2">
         <v>3</v>
@@ -3269,16 +4718,19 @@
       <c r="O44" s="2">
         <v>57.99</v>
       </c>
+      <c r="P44" t="s">
+        <v>306</v>
+      </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="C45" s="2" t="s">
         <v>238</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>239</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>30</v>
@@ -3287,25 +4739,25 @@
         <v>2019</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J45" s="2" t="s">
         <v>33</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M45" s="2">
         <v>4</v>
@@ -3316,16 +4768,19 @@
       <c r="O45" s="2">
         <v>58.99</v>
       </c>
+      <c r="P45" t="s">
+        <v>307</v>
+      </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="C46" s="2" t="s">
         <v>242</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>243</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>18</v>
@@ -3334,25 +4789,25 @@
         <v>2020</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J46" s="2" t="s">
         <v>33</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M46" s="2">
         <v>5</v>
@@ -3363,16 +4818,19 @@
       <c r="O46" s="2">
         <v>59.99</v>
       </c>
+      <c r="P46" t="s">
+        <v>308</v>
+      </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="C47" s="2" t="s">
         <v>246</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>247</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>30</v>
@@ -3387,19 +4845,19 @@
         <v>20</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J47" s="2" t="s">
         <v>23</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M47" s="2">
         <v>1</v>
@@ -3410,16 +4868,19 @@
       <c r="O47" s="2">
         <v>60.99</v>
       </c>
+      <c r="P47" t="s">
+        <v>309</v>
+      </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="C48" s="2" t="s">
         <v>250</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>251</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>18</v>
@@ -3434,19 +4895,19 @@
         <v>20</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J48" s="2" t="s">
         <v>33</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="M48" s="2">
         <v>2</v>
@@ -3457,16 +4918,19 @@
       <c r="O48" s="2">
         <v>61.99</v>
       </c>
+      <c r="P48" t="s">
+        <v>310</v>
+      </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>253</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>254</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>30</v>
@@ -3475,25 +4939,25 @@
         <v>2023</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J49" s="2" t="s">
         <v>33</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="M49" s="2">
         <v>3</v>
@@ -3504,16 +4968,19 @@
       <c r="O49" s="2">
         <v>62.99</v>
       </c>
+      <c r="P49" t="s">
+        <v>311</v>
+      </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="C50" s="2" t="s">
         <v>257</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>258</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>18</v>
@@ -3522,7 +4989,7 @@
         <v>2000</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>20</v>
@@ -3531,16 +4998,16 @@
         <v>21</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J50" s="2" t="s">
         <v>23</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="M50" s="2">
         <v>4</v>
@@ -3551,16 +5018,19 @@
       <c r="O50" s="2">
         <v>63.99</v>
       </c>
+      <c r="P50" t="s">
+        <v>312</v>
+      </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B51" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="C51" s="2" t="s">
         <v>261</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>262</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>30</v>
@@ -3569,7 +5039,7 @@
         <v>2001</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>20</v>
@@ -3578,16 +5048,16 @@
         <v>32</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J51" s="2" t="s">
         <v>33</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="M51" s="2">
         <v>5</v>
@@ -3597,6 +5067,9 @@
       </c>
       <c r="O51" s="2">
         <v>64.989999999999995</v>
+      </c>
+      <c r="P51" t="s">
+        <v>313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>